<commit_message>
build: se agrega mejora para menu
</commit_message>
<xml_diff>
--- a/documentos/Pruebas.xlsx
+++ b/documentos/Pruebas.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\personal\gestion-minimarket\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5B5AE6-59E9-44C8-9A8E-DBCF5BF37FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{011B6269-9088-4964-AAD6-B831101B6DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{90DC8E08-B72D-4FE1-934B-5D8DD9EE30BB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{90DC8E08-B72D-4FE1-934B-5D8DD9EE30BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Registro Producto" sheetId="7" r:id="rId1"/>
     <sheet name="Set de pruebas" sheetId="8" r:id="rId2"/>
     <sheet name="Prueba1" sheetId="9" r:id="rId3"/>
     <sheet name="Prueba_15122025" sheetId="10" r:id="rId4"/>
+    <sheet name="Hoja1" sheetId="11" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -145,7 +146,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="78">
   <si>
     <t>description</t>
   </si>
@@ -343,6 +344,42 @@
   </si>
   <si>
     <t>Se realiza la siguiente compra:</t>
+  </si>
+  <si>
+    <t>descripcion</t>
+  </si>
+  <si>
+    <t>Leche gloria tarro</t>
+  </si>
+  <si>
+    <t>Lata</t>
+  </si>
+  <si>
+    <t>Abarrotes</t>
+  </si>
+  <si>
+    <t>productstock</t>
+  </si>
+  <si>
+    <t>products</t>
+  </si>
+  <si>
+    <t>minimunStock</t>
+  </si>
+  <si>
+    <t>measures</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>abbreviation</t>
+  </si>
+  <si>
+    <t>unidad</t>
+  </si>
+  <si>
+    <t>kilo</t>
   </si>
 </sst>
 </file>
@@ -1762,4 +1799,131 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06FCA95E-8661-400A-BDD1-26CCDDD7D8FA}">
+  <dimension ref="A3:G16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="15.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
+        <v>1001</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="G5" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="1">
+        <v>1</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="1">
+        <v>2</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>